<commit_message>
update coordination reference file only, any unique geometry now has a unique generic PDB name
</commit_message>
<xml_diff>
--- a/wwpdb/utils/dp/metal/metal_ref/coord_classes_mapping_abbr.xlsx
+++ b/wwpdb/utils/dp/metal/metal_ref/coord_classes_mapping_abbr.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abiester/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81E9E0EB-BF0E-7648-9899-EA411A03BFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A28E89-ED9E-5649-B65B-223D88E4245F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9040" yWindow="760" windowWidth="25520" windowHeight="20280" tabRatio="215" xr2:uid="{CE4FFC7F-553B-A742-BB60-E7102764A25A}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="361">
   <si>
     <t>CN</t>
   </si>
@@ -650,21 +650,9 @@
     <t>square pyramidal with vacancy</t>
   </si>
   <si>
-    <t>pentagonal bipyramidal with vacancy</t>
-  </si>
-  <si>
-    <t>trigonal prismatic monocapped with vacancy</t>
-  </si>
-  <si>
     <t>trigonal prismatic monocapped</t>
   </si>
   <si>
-    <t>hexagonal bipyramidal with vacancy</t>
-  </si>
-  <si>
-    <t>octahedral monocapped</t>
-  </si>
-  <si>
     <t>square antiprismatic bicapped</t>
   </si>
   <si>
@@ -674,12 +662,6 @@
     <t>trigonal prism tricapped</t>
   </si>
   <si>
-    <t>octahedral bicapped</t>
-  </si>
-  <si>
-    <t>trigonal prismatic bicapped</t>
-  </si>
-  <si>
     <t>trigonal prismatic all face capped</t>
   </si>
   <si>
@@ -689,9 +671,6 @@
     <t>sandwich c5 5 i</t>
   </si>
   <si>
-    <t>octahedral monocapped with vacancy</t>
-  </si>
-  <si>
     <t>pyramidal</t>
   </si>
   <si>
@@ -1095,6 +1074,48 @@
   </si>
   <si>
     <t xml:space="preserve">trigonal prism square-face monocapped with a vacancy (non-capped edge)	</t>
+  </si>
+  <si>
+    <t>trigonal prismatic monocapped with capped face vacancy</t>
+  </si>
+  <si>
+    <t>trigonal prismatic monocapped with non-capped face vacancy</t>
+  </si>
+  <si>
+    <t>pentagonal bipyramidal with axial vacancy</t>
+  </si>
+  <si>
+    <t>octahedral monocapped with capped face vacancy</t>
+  </si>
+  <si>
+    <t>octahedral monocapped with non-capped face vacancy</t>
+  </si>
+  <si>
+    <t>hexagonal bipyramidal with axial vacancy</t>
+  </si>
+  <si>
+    <t>hexagonal bipyramidal with equatorial vacancy</t>
+  </si>
+  <si>
+    <t>pentagonal bipyramidal with equatorial vacancy</t>
+  </si>
+  <si>
+    <t>trigonal prismatic square-face bicapped</t>
+  </si>
+  <si>
+    <t>trigonal prismatic triangular-face bicapped</t>
+  </si>
+  <si>
+    <t>octahedral trans bicapped</t>
+  </si>
+  <si>
+    <t>octahedral cis bicapped</t>
+  </si>
+  <si>
+    <t>octahedral edge monocapped</t>
+  </si>
+  <si>
+    <t>octahedral face monocapped</t>
   </si>
 </sst>
 </file>
@@ -1546,13 +1567,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="C1" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="D1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="E1" t="s">
         <v>1</v>
@@ -1566,13 +1587,13 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="E2" t="s">
         <v>3</v>
@@ -1586,13 +1607,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="E3" t="s">
         <v>5</v>
@@ -1606,13 +1627,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E4" t="s">
         <v>7</v>
@@ -1626,19 +1647,19 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.15">
@@ -1646,13 +1667,13 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
@@ -1672,7 +1693,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="E7" t="s">
         <v>15</v>
@@ -1686,13 +1707,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C8" t="s">
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E8" t="s">
         <v>18</v>
@@ -1706,13 +1727,13 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="E9" t="s">
         <v>20</v>
@@ -1726,13 +1747,13 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="E10" t="s">
         <v>23</v>
@@ -1746,7 +1767,7 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C11" t="s">
         <v>25</v>
@@ -1766,7 +1787,7 @@
         <v>4</v>
       </c>
       <c r="B12" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="C12" t="s">
         <v>26</v>
@@ -1792,7 +1813,7 @@
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="E13" t="s">
         <v>27</v>
@@ -1812,7 +1833,7 @@
         <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -1832,13 +1853,13 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="E15" t="s">
         <v>31</v>
       </c>
       <c r="F15" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.15">
@@ -1846,13 +1867,13 @@
         <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C16" t="s">
         <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="E16" t="s">
         <v>33</v>
@@ -1866,13 +1887,13 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C17" t="s">
         <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E17" t="s">
         <v>36</v>
@@ -1886,7 +1907,7 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C18" t="s">
         <v>38</v>
@@ -1912,7 +1933,7 @@
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="E19" t="s">
         <v>40</v>
@@ -1932,7 +1953,7 @@
         <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="E20" t="s">
         <v>42</v>
@@ -1952,7 +1973,7 @@
         <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E21" t="s">
         <v>44</v>
@@ -1966,13 +1987,13 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="C22" t="s">
         <v>46</v>
       </c>
       <c r="D22" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="E22" t="s">
         <v>47</v>
@@ -1986,13 +2007,13 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C23" t="s">
         <v>48</v>
       </c>
       <c r="D23" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="E23" t="s">
         <v>49</v>
@@ -2006,7 +2027,7 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C24" t="s">
         <v>51</v>
@@ -2018,7 +2039,7 @@
         <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>205</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.15">
@@ -2026,7 +2047,7 @@
         <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C25" t="s">
         <v>52</v>
@@ -2038,7 +2059,7 @@
         <v>14</v>
       </c>
       <c r="F25" t="s">
-        <v>205</v>
+        <v>354</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.15">
@@ -2046,10 +2067,10 @@
         <v>6</v>
       </c>
       <c r="B26" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C26" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="D26" t="s">
         <v>14</v>
@@ -2058,7 +2079,7 @@
         <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>218</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.15">
@@ -2066,10 +2087,10 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="C27" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="D27" t="s">
         <v>14</v>
@@ -2078,7 +2099,7 @@
         <v>14</v>
       </c>
       <c r="F27" t="s">
-        <v>218</v>
+        <v>351</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.15">
@@ -2086,10 +2107,10 @@
         <v>6</v>
       </c>
       <c r="B28" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C28" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="D28" t="s">
         <v>14</v>
@@ -2098,7 +2119,7 @@
         <v>14</v>
       </c>
       <c r="F28" t="s">
-        <v>206</v>
+        <v>347</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.15">
@@ -2106,10 +2127,10 @@
         <v>6</v>
       </c>
       <c r="B29" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="C29" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="D29" t="s">
         <v>14</v>
@@ -2118,7 +2139,7 @@
         <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>206</v>
+        <v>348</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.15">
@@ -2132,7 +2153,7 @@
         <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="E30" t="s">
         <v>53</v>
@@ -2152,7 +2173,7 @@
         <v>14</v>
       </c>
       <c r="D31" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="E31" t="s">
         <v>55</v>
@@ -2172,7 +2193,7 @@
         <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="E32" t="s">
         <v>57</v>
@@ -2192,7 +2213,7 @@
         <v>14</v>
       </c>
       <c r="D33" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="E33" t="s">
         <v>59</v>
@@ -2212,7 +2233,7 @@
         <v>14</v>
       </c>
       <c r="D34" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="E34" t="s">
         <v>61</v>
@@ -2226,13 +2247,13 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="C35" t="s">
         <v>63</v>
       </c>
       <c r="D35" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="E35" t="s">
         <v>64</v>
@@ -2246,19 +2267,19 @@
         <v>7</v>
       </c>
       <c r="B36" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C36" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="D36" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="E36" t="s">
         <v>66</v>
       </c>
       <c r="F36" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.15">
@@ -2266,10 +2287,10 @@
         <v>7</v>
       </c>
       <c r="B37" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C37" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="D37" t="s">
         <v>14</v>
@@ -2278,7 +2299,7 @@
         <v>14</v>
       </c>
       <c r="F37" t="s">
-        <v>209</v>
+        <v>360</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.15">
@@ -2286,7 +2307,7 @@
         <v>7</v>
       </c>
       <c r="B38" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C38" t="s">
         <v>67</v>
@@ -2298,7 +2319,7 @@
         <v>14</v>
       </c>
       <c r="F38" t="s">
-        <v>208</v>
+        <v>352</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.15">
@@ -2306,7 +2327,7 @@
         <v>7</v>
       </c>
       <c r="B39" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C39" t="s">
         <v>68</v>
@@ -2318,7 +2339,7 @@
         <v>14</v>
       </c>
       <c r="F39" t="s">
-        <v>208</v>
+        <v>353</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.15">
@@ -2326,7 +2347,7 @@
         <v>7</v>
       </c>
       <c r="B40" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C40" t="s">
         <v>69</v>
@@ -2346,7 +2367,7 @@
         <v>7</v>
       </c>
       <c r="B41" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C41" t="s">
         <v>71</v>
@@ -2372,13 +2393,13 @@
         <v>14</v>
       </c>
       <c r="D42" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="E42" t="s">
         <v>73</v>
       </c>
       <c r="F42" t="s">
-        <v>209</v>
+        <v>359</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.15">
@@ -2392,7 +2413,7 @@
         <v>14</v>
       </c>
       <c r="D43" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="E43" t="s">
         <v>74</v>
@@ -2412,7 +2433,7 @@
         <v>14</v>
       </c>
       <c r="D44" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="E44" t="s">
         <v>76</v>
@@ -2432,7 +2453,7 @@
         <v>14</v>
       </c>
       <c r="D45" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="E45" t="s">
         <v>78</v>
@@ -2452,7 +2473,7 @@
         <v>14</v>
       </c>
       <c r="D46" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="E46" t="s">
         <v>80</v>
@@ -2466,13 +2487,13 @@
         <v>8</v>
       </c>
       <c r="B47" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="C47" t="s">
         <v>82</v>
       </c>
       <c r="D47" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="E47" t="s">
         <v>83</v>
@@ -2486,13 +2507,13 @@
         <v>8</v>
       </c>
       <c r="B48" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="C48" t="s">
         <v>85</v>
       </c>
       <c r="D48" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="E48" t="s">
         <v>86</v>
@@ -2506,13 +2527,13 @@
         <v>8</v>
       </c>
       <c r="B49" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="C49" t="s">
         <v>87</v>
       </c>
       <c r="D49" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E49" t="s">
         <v>88</v>
@@ -2526,10 +2547,10 @@
         <v>8</v>
       </c>
       <c r="B50" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="C50" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="D50" t="s">
         <v>14</v>
@@ -2538,7 +2559,7 @@
         <v>14</v>
       </c>
       <c r="F50" t="s">
-        <v>213</v>
+        <v>357</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.15">
@@ -2546,10 +2567,10 @@
         <v>8</v>
       </c>
       <c r="B51" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="C51" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="D51" t="s">
         <v>14</v>
@@ -2558,7 +2579,7 @@
         <v>14</v>
       </c>
       <c r="F51" t="s">
-        <v>214</v>
+        <v>355</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.15">
@@ -2566,19 +2587,19 @@
         <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C52" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="D52" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="E52" t="s">
         <v>90</v>
       </c>
       <c r="F52" t="s">
-        <v>214</v>
+        <v>356</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.15">
@@ -2592,7 +2613,7 @@
         <v>14</v>
       </c>
       <c r="D53" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="E53" t="s">
         <v>91</v>
@@ -2612,7 +2633,7 @@
         <v>14</v>
       </c>
       <c r="D54" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E54" t="s">
         <v>93</v>
@@ -2632,7 +2653,7 @@
         <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="E55" t="s">
         <v>95</v>
@@ -2652,7 +2673,7 @@
         <v>14</v>
       </c>
       <c r="D56" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="E56" t="s">
         <v>97</v>
@@ -2672,7 +2693,7 @@
         <v>14</v>
       </c>
       <c r="D57" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="E57" t="s">
         <v>99</v>
@@ -2692,7 +2713,7 @@
         <v>14</v>
       </c>
       <c r="D58" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="E58" t="s">
         <v>101</v>
@@ -2712,13 +2733,13 @@
         <v>14</v>
       </c>
       <c r="D59" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="E59" t="s">
         <v>103</v>
       </c>
       <c r="F59" t="s">
-        <v>213</v>
+        <v>358</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.15">
@@ -2732,7 +2753,7 @@
         <v>14</v>
       </c>
       <c r="D60" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="E60" t="s">
         <v>104</v>
@@ -2752,7 +2773,7 @@
         <v>14</v>
       </c>
       <c r="D61" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="E61" t="s">
         <v>106</v>
@@ -2766,19 +2787,19 @@
         <v>9</v>
       </c>
       <c r="B62" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="C62" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="D62" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="E62" t="s">
         <v>107</v>
       </c>
       <c r="F62" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
@@ -2786,10 +2807,10 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="C63" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="D63" t="s">
         <v>14</v>
@@ -2798,7 +2819,7 @@
         <v>14</v>
       </c>
       <c r="F63" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.15">
@@ -2812,7 +2833,7 @@
         <v>14</v>
       </c>
       <c r="D64" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="E64" t="s">
         <v>108</v>
@@ -2832,7 +2853,7 @@
         <v>14</v>
       </c>
       <c r="D65" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="E65" t="s">
         <v>110</v>
@@ -2852,7 +2873,7 @@
         <v>14</v>
       </c>
       <c r="D66" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="E66" t="s">
         <v>112</v>
@@ -2872,7 +2893,7 @@
         <v>14</v>
       </c>
       <c r="D67" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="E67" t="s">
         <v>114</v>
@@ -2892,7 +2913,7 @@
         <v>14</v>
       </c>
       <c r="D68" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="E68" t="s">
         <v>116</v>
@@ -2912,7 +2933,7 @@
         <v>14</v>
       </c>
       <c r="D69" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E69" t="s">
         <v>118</v>
@@ -2932,13 +2953,13 @@
         <v>14</v>
       </c>
       <c r="D70" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="E70" t="s">
         <v>120</v>
       </c>
       <c r="F70" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.15">
@@ -2952,7 +2973,7 @@
         <v>14</v>
       </c>
       <c r="D71" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="E71" t="s">
         <v>121</v>
@@ -2972,7 +2993,7 @@
         <v>14</v>
       </c>
       <c r="D72" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="E72" t="s">
         <v>123</v>
@@ -2992,7 +3013,7 @@
         <v>14</v>
       </c>
       <c r="D73" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="E73" t="s">
         <v>125</v>
@@ -3012,7 +3033,7 @@
         <v>14</v>
       </c>
       <c r="D74" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="E74" t="s">
         <v>127</v>
@@ -3032,7 +3053,7 @@
         <v>14</v>
       </c>
       <c r="D75" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="E75" t="s">
         <v>129</v>
@@ -3052,7 +3073,7 @@
         <v>14</v>
       </c>
       <c r="D76" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="E76" t="s">
         <v>131</v>
@@ -3072,7 +3093,7 @@
         <v>14</v>
       </c>
       <c r="D77" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="E77" t="s">
         <v>133</v>
@@ -3092,7 +3113,7 @@
         <v>14</v>
       </c>
       <c r="D78" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="E78" t="s">
         <v>135</v>
@@ -3112,7 +3133,7 @@
         <v>14</v>
       </c>
       <c r="D79" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="E79" t="s">
         <v>137</v>
@@ -3132,7 +3153,7 @@
         <v>14</v>
       </c>
       <c r="D80" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="E80" t="s">
         <v>139</v>
@@ -3152,13 +3173,13 @@
         <v>14</v>
       </c>
       <c r="D81" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="E81" t="s">
         <v>141</v>
       </c>
       <c r="F81" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.15">
@@ -3172,7 +3193,7 @@
         <v>14</v>
       </c>
       <c r="D82" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="E82" t="s">
         <v>142</v>
@@ -3192,7 +3213,7 @@
         <v>14</v>
       </c>
       <c r="D83" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="E83" t="s">
         <v>144</v>
@@ -3212,7 +3233,7 @@
         <v>14</v>
       </c>
       <c r="D84" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="E84" t="s">
         <v>146</v>
@@ -3232,7 +3253,7 @@
         <v>14</v>
       </c>
       <c r="D85" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="E85" t="s">
         <v>148</v>
@@ -3252,7 +3273,7 @@
         <v>14</v>
       </c>
       <c r="D86" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="E86" t="s">
         <v>150</v>
@@ -3272,7 +3293,7 @@
         <v>14</v>
       </c>
       <c r="D87" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="E87" t="s">
         <v>152</v>
@@ -3292,7 +3313,7 @@
         <v>14</v>
       </c>
       <c r="D88" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="E88" t="s">
         <v>154</v>
@@ -3312,7 +3333,7 @@
         <v>14</v>
       </c>
       <c r="D89" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="E89" t="s">
         <v>156</v>
@@ -3332,7 +3353,7 @@
         <v>14</v>
       </c>
       <c r="D90" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="E90" t="s">
         <v>158</v>
@@ -3352,7 +3373,7 @@
         <v>14</v>
       </c>
       <c r="D91" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="E91" t="s">
         <v>160</v>
@@ -3372,7 +3393,7 @@
         <v>14</v>
       </c>
       <c r="D92" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="E92" t="s">
         <v>162</v>
@@ -3392,7 +3413,7 @@
         <v>14</v>
       </c>
       <c r="D93" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E93" t="s">
         <v>164</v>
@@ -3412,7 +3433,7 @@
         <v>14</v>
       </c>
       <c r="D94" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="E94" t="s">
         <v>166</v>
@@ -3432,7 +3453,7 @@
         <v>14</v>
       </c>
       <c r="D95" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="E95" t="s">
         <v>168</v>
@@ -3452,7 +3473,7 @@
         <v>14</v>
       </c>
       <c r="D96" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="E96" t="s">
         <v>170</v>
@@ -3472,7 +3493,7 @@
         <v>14</v>
       </c>
       <c r="D97" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="E97" t="s">
         <v>172</v>
@@ -3492,7 +3513,7 @@
         <v>14</v>
       </c>
       <c r="D98" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="E98" t="s">
         <v>174</v>
@@ -3512,7 +3533,7 @@
         <v>14</v>
       </c>
       <c r="D99" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="E99" t="s">
         <v>176</v>
@@ -3532,13 +3553,13 @@
         <v>14</v>
       </c>
       <c r="D100" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="E100" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="F100" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.15">
@@ -3552,7 +3573,7 @@
         <v>14</v>
       </c>
       <c r="D101" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="E101" t="s">
         <v>178</v>
@@ -3572,7 +3593,7 @@
         <v>14</v>
       </c>
       <c r="D102" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="E102" t="s">
         <v>180</v>
@@ -3592,7 +3613,7 @@
         <v>14</v>
       </c>
       <c r="D103" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="E103" t="s">
         <v>182</v>
@@ -3612,7 +3633,7 @@
         <v>14</v>
       </c>
       <c r="D104" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="E104" t="s">
         <v>184</v>
@@ -3632,7 +3653,7 @@
         <v>14</v>
       </c>
       <c r="D105" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="E105" t="s">
         <v>186</v>
@@ -3652,7 +3673,7 @@
         <v>14</v>
       </c>
       <c r="D106" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E106" t="s">
         <v>188</v>
@@ -3672,7 +3693,7 @@
         <v>14</v>
       </c>
       <c r="D107" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="E107" t="s">
         <v>190</v>
@@ -3692,7 +3713,7 @@
         <v>14</v>
       </c>
       <c r="D108" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E108" t="s">
         <v>192</v>
@@ -3712,7 +3733,7 @@
         <v>14</v>
       </c>
       <c r="D109" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="E109" t="s">
         <v>194</v>
@@ -3732,7 +3753,7 @@
         <v>14</v>
       </c>
       <c r="D110" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="E110" t="s">
         <v>196</v>
@@ -3752,7 +3773,7 @@
         <v>14</v>
       </c>
       <c r="D111" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="E111" t="s">
         <v>198</v>
@@ -3772,7 +3793,7 @@
         <v>14</v>
       </c>
       <c r="D112" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="E112" t="s">
         <v>200</v>
@@ -3792,7 +3813,7 @@
         <v>14</v>
       </c>
       <c r="D113" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="E113" t="s">
         <v>202</v>
@@ -3809,7 +3830,7 @@
         <v>14</v>
       </c>
       <c r="C114" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D114" t="s">
         <v>14</v>
@@ -3818,7 +3839,7 @@
         <v>14</v>
       </c>
       <c r="F114" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>